<commit_message>
Enermech and Saipem added succesfully
</commit_message>
<xml_diff>
--- a/data/input/master_companies_with_fingerprint.xlsx
+++ b/data/input/master_companies_with_fingerprint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alirizabagci/Documents/Python Projects/Upwork/Singapore_ATS_Scraping_Delivery_batch2/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E6B3622-48EE-2447-9497-85EBB76F763A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{926914C4-8D67-3F4E-B36E-F32A65C69622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1959" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1964" uniqueCount="303">
   <si>
     <t>Company</t>
   </si>
@@ -922,6 +922,21 @@
   </si>
   <si>
     <t>carrier_html</t>
+  </si>
+  <si>
+    <t>Enermech</t>
+  </si>
+  <si>
+    <t>https://apply.workable.com/enermech/</t>
+  </si>
+  <si>
+    <t>enermech_workable</t>
+  </si>
+  <si>
+    <t>https://jobs.saipem.com/</t>
+  </si>
+  <si>
+    <t>saipem_ncore</t>
   </si>
 </sst>
 </file>
@@ -1385,7 +1400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O66"/>
+  <dimension ref="A1:O67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="255.83203125" bestFit="1" customWidth="1"/>
@@ -2778,6 +2793,9 @@
       <c r="D32" s="7" t="s">
         <v>152</v>
       </c>
+      <c r="E32" s="16" t="s">
+        <v>301</v>
+      </c>
       <c r="G32" s="6" t="s">
         <v>77</v>
       </c>
@@ -2788,7 +2806,7 @@
         <v>78</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>77</v>
+        <v>302</v>
       </c>
       <c r="M32" s="6" t="b">
         <v>1</v>
@@ -4300,6 +4318,20 @@
       </c>
       <c r="O66" s="12" t="s">
         <v>274</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A67" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="D67" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="E67" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="L67" s="12" t="s">
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -4354,6 +4386,9 @@
     <hyperlink ref="E65" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
     <hyperlink ref="E66" r:id="rId48" location="component__content-set-2" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
     <hyperlink ref="D49" r:id="rId49" xr:uid="{C83E8530-7B63-7546-80DE-6A2E917C99F4}"/>
+    <hyperlink ref="E67" r:id="rId50" xr:uid="{8D9B298E-C4AE-EA44-A0F9-7E0745BEBC02}"/>
+    <hyperlink ref="E32" r:id="rId51" xr:uid="{0F133174-28D9-5649-BB96-F9970F0DCC5A}"/>
+    <hyperlink ref="D67" r:id="rId52" xr:uid="{7250D070-7E5C-5B49-BD9A-ECE70091B1FB}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Fix utf-8 excel bug
</commit_message>
<xml_diff>
--- a/data/input/master_companies_with_fingerprint.xlsx
+++ b/data/input/master_companies_with_fingerprint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alirizabagci/Documents/Python Projects/Upwork/Singapore_ATS_Scraping_Delivery_batch2/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{926914C4-8D67-3F4E-B36E-F32A65C69622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{216FC8ED-0CE6-444C-B045-C5C450B979C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1964" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1965" uniqueCount="304">
   <si>
     <t>Company</t>
   </si>
@@ -937,6 +937,9 @@
   </si>
   <si>
     <t>saipem_ncore</t>
+  </si>
+  <si>
+    <t>clinch_careers_site</t>
   </si>
 </sst>
 </file>
@@ -2849,6 +2852,9 @@
       <c r="K33" s="17" t="s">
         <v>42</v>
       </c>
+      <c r="L33" s="17" t="s">
+        <v>303</v>
+      </c>
       <c r="M33" s="17" t="b">
         <v>1</v>
       </c>
@@ -3032,50 +3038,50 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:15" s="17" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="17" t="s">
+    <row r="38" spans="1:15" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="B38" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C38" s="17">
+      <c r="B38" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" s="12">
         <v>137</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="D38" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="E38" s="18" t="s">
+      <c r="E38" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="F38" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="G38" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="H38" s="17" t="s">
+      <c r="F38" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G38" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="H38" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="I38" s="17" t="s">
+      <c r="I38" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="J38" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="K38" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="L38" s="17" t="s">
+      <c r="J38" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="K38" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="L38" s="12" t="s">
         <v>296</v>
       </c>
-      <c r="M38" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="N38" s="17" t="s">
+      <c r="M38" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="N38" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="O38" s="17" t="s">
+      <c r="O38" s="12" t="s">
         <v>174</v>
       </c>
     </row>

</xml_diff>